<commit_message>
Withdraw the Bayesian path ranking (owner decision); publish reconciled path status instead
Root cause: the scorer looked paths up as 'A -> B' in a store keyed 'A_B', so
validation never applied (all 48 paths NOT_VALIDATED since 2026-03-20); its
counts were regex artefacts; a recompute read a field renamed on 2026-08-21.
The Statistical Analysis page now shows each path's reconciled status, live
evidence count and study design, explicitly not a ranking. Contradicted paths
are counted, not named (suppression gate). posterioragree stage retired.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Analysis/Results/literature_gap_matrix.xlsx
+++ b/Analysis/Results/literature_gap_matrix.xlsx
@@ -2155,7 +2155,7 @@
         <v>18</v>
       </c>
       <c r="T16" s="6" t="n">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="U16" s="6" t="n">
         <v>667</v>
@@ -2185,7 +2185,7 @@
         <v>543</v>
       </c>
       <c r="AD16" s="10" t="n">
-        <v>2750</v>
+        <v>2751</v>
       </c>
       <c r="AE16" s="6" t="n">
         <v>234</v>
@@ -2349,7 +2349,7 @@
         <v>51</v>
       </c>
       <c r="T18" s="10" t="n">
-        <v>2111</v>
+        <v>2112</v>
       </c>
       <c r="U18" s="6" t="n">
         <v>531</v>
@@ -2379,7 +2379,7 @@
         <v>360</v>
       </c>
       <c r="AD18" s="10" t="n">
-        <v>2419</v>
+        <v>2422</v>
       </c>
       <c r="AE18" s="5" t="n">
         <v>58</v>
@@ -2476,7 +2476,7 @@
         <v>2</v>
       </c>
       <c r="AD19" s="5" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="AE19" s="7" t="n">
         <v>10</v>
@@ -2531,13 +2531,13 @@
         <v>223</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="Q20" s="5" t="n">
         <v>81</v>
       </c>
       <c r="R20" s="10" t="n">
-        <v>2111</v>
+        <v>2112</v>
       </c>
       <c r="S20" s="7" t="n">
         <v>16</v>
@@ -2573,10 +2573,10 @@
         <v>49</v>
       </c>
       <c r="AD20" s="10" t="n">
-        <v>2996</v>
+        <v>2997</v>
       </c>
       <c r="AE20" s="5" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21">
@@ -2649,13 +2649,13 @@
         <v>318</v>
       </c>
       <c r="W21" s="10" t="n">
-        <v>1323</v>
+        <v>1325</v>
       </c>
       <c r="X21" s="7" t="n">
         <v>10</v>
       </c>
       <c r="Y21" s="5" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Z21" s="7" t="n">
         <v>15</v>
@@ -2670,7 +2670,7 @@
         <v>24</v>
       </c>
       <c r="AD21" s="10" t="n">
-        <v>2869</v>
+        <v>2870</v>
       </c>
       <c r="AE21" s="5" t="n">
         <v>135</v>
@@ -2837,7 +2837,7 @@
         <v>636</v>
       </c>
       <c r="U23" s="10" t="n">
-        <v>1323</v>
+        <v>1325</v>
       </c>
       <c r="V23" s="6" t="n">
         <v>256</v>
@@ -2864,7 +2864,7 @@
         <v>677</v>
       </c>
       <c r="AD23" s="10" t="n">
-        <v>8324</v>
+        <v>8326</v>
       </c>
       <c r="AE23" s="6" t="n">
         <v>382</v>
@@ -2946,7 +2946,7 @@
         <v>1987</v>
       </c>
       <c r="Y24" s="6" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="Z24" s="7" t="n">
         <v>13</v>
@@ -3031,7 +3031,7 @@
         <v>91</v>
       </c>
       <c r="U25" s="5" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V25" s="7" t="n">
         <v>18</v>
@@ -3040,7 +3040,7 @@
         <v>254</v>
       </c>
       <c r="X25" s="6" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="Y25" s="4" t="n">
         <v>7108</v>
@@ -3252,7 +3252,7 @@
         <v>329</v>
       </c>
       <c r="AD27" s="10" t="n">
-        <v>2164</v>
+        <v>2165</v>
       </c>
       <c r="AE27" s="6" t="n">
         <v>285</v>
@@ -3501,28 +3501,28 @@
         <v>881</v>
       </c>
       <c r="P30" s="10" t="n">
-        <v>2750</v>
+        <v>2751</v>
       </c>
       <c r="Q30" s="6" t="n">
         <v>389</v>
       </c>
       <c r="R30" s="10" t="n">
-        <v>2419</v>
+        <v>2422</v>
       </c>
       <c r="S30" s="5" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="T30" s="10" t="n">
-        <v>2996</v>
+        <v>2997</v>
       </c>
       <c r="U30" s="10" t="n">
-        <v>2869</v>
+        <v>2870</v>
       </c>
       <c r="V30" s="6" t="n">
         <v>579</v>
       </c>
       <c r="W30" s="10" t="n">
-        <v>8324</v>
+        <v>8326</v>
       </c>
       <c r="X30" s="6" t="n">
         <v>325</v>
@@ -3534,7 +3534,7 @@
         <v>735</v>
       </c>
       <c r="AA30" s="10" t="n">
-        <v>2164</v>
+        <v>2165</v>
       </c>
       <c r="AB30" s="7" t="n">
         <v>46</v>
@@ -3610,7 +3610,7 @@
         <v>10</v>
       </c>
       <c r="T31" s="5" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="U31" s="5" t="n">
         <v>135</v>
@@ -9406,7 +9406,7 @@
         <v>99.40000000000001</v>
       </c>
       <c r="E164" s="12" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F164" s="12" t="n">
         <v>10198.6</v>
@@ -10141,7 +10141,7 @@
         <v>99.3</v>
       </c>
       <c r="E185" s="12" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F185" s="12" t="n">
         <v>8818.9</v>
@@ -13524,28 +13524,28 @@
       </c>
       <c r="B282" s="12" t="inlineStr">
         <is>
-          <t>Drug Repurposing</t>
+          <t>CV Complications</t>
         </is>
       </c>
       <c r="C282" s="12" t="inlineStr">
         <is>
-          <t>Prevention / DPP</t>
+          <t>CGM Technology</t>
         </is>
       </c>
       <c r="D282" s="12" t="n">
         <v>98.2</v>
       </c>
       <c r="E282" s="12" t="n">
-        <v>133</v>
+        <v>254</v>
       </c>
       <c r="F282" s="12" t="n">
-        <v>7191.1</v>
+        <v>13780.1</v>
       </c>
       <c r="G282" s="12" t="n">
-        <v>625</v>
+        <v>26715</v>
       </c>
       <c r="H282" s="12" t="n">
-        <v>82739</v>
+        <v>7108</v>
       </c>
       <c r="I282" s="13" t="inlineStr">
         <is>
@@ -13559,28 +13559,28 @@
       </c>
       <c r="B283" s="12" t="inlineStr">
         <is>
-          <t>CV Complications</t>
+          <t>Epigenetics</t>
         </is>
       </c>
       <c r="C283" s="12" t="inlineStr">
         <is>
-          <t>CGM Technology</t>
+          <t>AI / ML Predict</t>
         </is>
       </c>
       <c r="D283" s="12" t="n">
-        <v>98.2</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="E283" s="12" t="n">
-        <v>254</v>
+        <v>190</v>
       </c>
       <c r="F283" s="12" t="n">
-        <v>13780.1</v>
+        <v>9778.200000000001</v>
       </c>
       <c r="G283" s="12" t="n">
-        <v>26715</v>
+        <v>7861</v>
       </c>
       <c r="H283" s="12" t="n">
-        <v>7108</v>
+        <v>12163</v>
       </c>
       <c r="I283" s="13" t="inlineStr">
         <is>
@@ -13594,28 +13594,28 @@
       </c>
       <c r="B284" s="12" t="inlineStr">
         <is>
-          <t>Epigenetics</t>
+          <t>GLP-1 Agonists</t>
         </is>
       </c>
       <c r="C284" s="12" t="inlineStr">
         <is>
-          <t>AI / ML Predict</t>
+          <t>Drug Repurposing</t>
         </is>
       </c>
       <c r="D284" s="12" t="n">
         <v>98.09999999999999</v>
       </c>
       <c r="E284" s="12" t="n">
-        <v>190</v>
+        <v>56</v>
       </c>
       <c r="F284" s="12" t="n">
-        <v>9778.200000000001</v>
+        <v>2961.3</v>
       </c>
       <c r="G284" s="12" t="n">
-        <v>7861</v>
+        <v>14031</v>
       </c>
       <c r="H284" s="12" t="n">
-        <v>12163</v>
+        <v>625</v>
       </c>
       <c r="I284" s="13" t="inlineStr">
         <is>
@@ -13634,23 +13634,23 @@
       </c>
       <c r="C285" s="12" t="inlineStr">
         <is>
-          <t>Drug Repurposing</t>
+          <t>CGM Technology</t>
         </is>
       </c>
       <c r="D285" s="12" t="n">
         <v>98.09999999999999</v>
       </c>
       <c r="E285" s="12" t="n">
-        <v>56</v>
+        <v>187</v>
       </c>
       <c r="F285" s="12" t="n">
-        <v>2961.3</v>
+        <v>9986.6</v>
       </c>
       <c r="G285" s="12" t="n">
         <v>14031</v>
       </c>
       <c r="H285" s="12" t="n">
-        <v>625</v>
+        <v>7108</v>
       </c>
       <c r="I285" s="13" t="inlineStr">
         <is>
@@ -13664,28 +13664,28 @@
       </c>
       <c r="B286" s="12" t="inlineStr">
         <is>
-          <t>GLP-1 Agonists</t>
+          <t>Multi-Omics</t>
         </is>
       </c>
       <c r="C286" s="12" t="inlineStr">
         <is>
-          <t>CGM Technology</t>
+          <t>Drug Repurposing</t>
         </is>
       </c>
       <c r="D286" s="12" t="n">
         <v>98.09999999999999</v>
       </c>
       <c r="E286" s="12" t="n">
-        <v>187</v>
+        <v>21</v>
       </c>
       <c r="F286" s="12" t="n">
-        <v>9986.6</v>
+        <v>1096.3</v>
       </c>
       <c r="G286" s="12" t="n">
-        <v>14031</v>
+        <v>1923</v>
       </c>
       <c r="H286" s="12" t="n">
-        <v>7108</v>
+        <v>625</v>
       </c>
       <c r="I286" s="13" t="inlineStr">
         <is>
@@ -13699,28 +13699,28 @@
       </c>
       <c r="B287" s="12" t="inlineStr">
         <is>
-          <t>Multi-Omics</t>
+          <t>Drug Repurposing</t>
         </is>
       </c>
       <c r="C287" s="12" t="inlineStr">
         <is>
-          <t>Drug Repurposing</t>
+          <t>Prevention / DPP</t>
         </is>
       </c>
       <c r="D287" s="12" t="n">
         <v>98.09999999999999</v>
       </c>
       <c r="E287" s="12" t="n">
-        <v>21</v>
+        <v>134</v>
       </c>
       <c r="F287" s="12" t="n">
-        <v>1096.3</v>
+        <v>7191.1</v>
       </c>
       <c r="G287" s="12" t="n">
-        <v>1923</v>
+        <v>625</v>
       </c>
       <c r="H287" s="12" t="n">
-        <v>625</v>
+        <v>82739</v>
       </c>
       <c r="I287" s="13" t="inlineStr">
         <is>
@@ -14376,7 +14376,7 @@
         <v>97.7</v>
       </c>
       <c r="E306" s="12" t="n">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F306" s="12" t="n">
         <v>15040.2</v>
@@ -17841,7 +17841,7 @@
         <v>93.3</v>
       </c>
       <c r="E405" s="12" t="n">
-        <v>1323</v>
+        <v>1325</v>
       </c>
       <c r="F405" s="12" t="n">
         <v>19771.7</v>
@@ -18051,7 +18051,7 @@
         <v>92.40000000000001</v>
       </c>
       <c r="E411" s="12" t="n">
-        <v>2419</v>
+        <v>2422</v>
       </c>
       <c r="F411" s="12" t="n">
         <v>31723.1</v>
@@ -18156,7 +18156,7 @@
         <v>92.09999999999999</v>
       </c>
       <c r="E414" s="12" t="n">
-        <v>2996</v>
+        <v>2997</v>
       </c>
       <c r="F414" s="12" t="n">
         <v>37979.9</v>
@@ -18226,7 +18226,7 @@
         <v>91.8</v>
       </c>
       <c r="E416" s="12" t="n">
-        <v>2869</v>
+        <v>2870</v>
       </c>
       <c r="F416" s="12" t="n">
         <v>34795.4</v>
@@ -18296,7 +18296,7 @@
         <v>91.7</v>
       </c>
       <c r="E418" s="12" t="n">
-        <v>2164</v>
+        <v>2165</v>
       </c>
       <c r="F418" s="12" t="n">
         <v>26106</v>
@@ -18331,7 +18331,7 @@
         <v>91.59999999999999</v>
       </c>
       <c r="E419" s="12" t="n">
-        <v>2750</v>
+        <v>2751</v>
       </c>
       <c r="F419" s="12" t="n">
         <v>32764.9</v>
@@ -18681,7 +18681,7 @@
         <v>85.5</v>
       </c>
       <c r="E429" s="12" t="n">
-        <v>2111</v>
+        <v>2112</v>
       </c>
       <c r="F429" s="12" t="n">
         <v>14561.9</v>
@@ -18856,7 +18856,7 @@
         <v>82.3</v>
       </c>
       <c r="E434" s="12" t="n">
-        <v>8324</v>
+        <v>8326</v>
       </c>
       <c r="F434" s="12" t="n">
         <v>47014.6</v>
@@ -18891,7 +18891,7 @@
         <v>80</v>
       </c>
       <c r="E435" s="12" t="n">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="F435" s="12" t="n">
         <v>3758.1</v>

</xml_diff>